<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-03 La petite voiture verte
Réécriture vocale example4 : éclat de rond, parle peu vécu.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-03.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-03.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La maison au bout du tapis</t>
+          <t>La petite voiture verte</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>entrée mouillée, classe, puis parc</t>
+          <t>école puis parc : casiers, manteau, vitre embuée, voiture verte, sable, seau</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut que la voiture verte arrive à la maison de cubes. Aniss parle peu. Elle lui tend la voiture. Plus tard au parc, elle lui tend un seau. Ils font un chemin de sable.</t>
+          <t>Un petit rond de doigt s'ouvre sur la vitre. Au bord, un éclat de rond brille. Mila veut jouer à la voiture, maintenant. Elle pose trop de questions. Aniss se tait, recule. Sourire parti, poitrine, papa accroupi. Elle refuse de foncer, referme la bouche, tend la voiture, attend. Merci vécu. Au parc, seau trop vite. Un éclat de rond tient au bord.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe du manteau rouge. Elle fait un rond sombre sur le carrelage. Le manteau sent encore la pluie. Les casiers sont un peu froids. Un cartable frotte le bois. Papa noue les lacets de Mila. Les lacets font un bruit de tissu. Tu as ton goûter dans la poche. Les lacets sont bien faits ? Oui, papa. Un cube jaune attend sur le tapis. Puis un cube bleu. Le tapis sent un peu la laine. En ce moment, Mila pose les cubes. Le cube jaune est lisse. Je fais une maison. Pour la voiture verte. Une maison au bout du tapis ? Oui. Elle doit arriver. Aniss arrive. Aniss parle peu. Il regarde le tapis. Mila a envie de poser beaucoup de questions. Elle referme un peu la bouche. On peut attendre. Tu peux tendre un jouet. La voiture verte est dans sa main. Les roues sont lisses. Aniss ne dit rien.</t>
+          <t>La fermeture du manteau rouge accroche un casier. Elle tient, papa. Tu la tires, Mila ? Oui, il est froid. Papa libère la fermeture, d'un coup. Une goutte saute sur la vitre. Elle est ronde. Tu as vu la goutte, Mila ? Oui, maman. La vitre est embuée, un peu. Mila pose un doigt au milieu. Un petit rond s'ouvre, net. Au bord, un éclat de rond brille. Il brille, papa. Tu le vois, ce petit point ? Oui, un petit point. Les casiers sentent le bois mouillé. Ça sent la pluie, maman. Le goûter est dans la poche ? Oui, maman. Le bois du casier est froid, sous la paume. Il pique un peu. Tes doigts sont froids, Mila ? Un peu, papa. Un cube jaune attend sur le tapis. Puis un cube bleu, plus loin. Ils sont lisses. Le tapis est prêt, Mila ? Oui, papa. En ce moment, Mila pose les cubes. Je veux jouer à la voiture, maintenant ! Pour la maison, au bout du tapis. Une maison au bout du tapis ? Oui. Elle doit arriver tout de suite. La voiture verte est dans sa main. Les roues sont lisses, un peu froides. Aniss arrive près du tapis. Il s'arrête, sans parler. Tu viens, Aniss ? On fait la maison ? Tu prends la voiture ? Les questions tombent trop vite. Prends-la ! Mila tend la voiture trop vite. Aniss recule d'un pas. Ses épaules se serrent. Il ne dit rien. Aniss ? Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Mila ? Oui, papa. Tes mains tiennent la voiture, Mila ? Un peu, maman. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le petit rond, un instant. L'éclat de rond tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur la vitre.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une goutte tombe du manteau rouge. Elle fait un rond sombre sur le carrelage. Le manteau sent encore la pluie. Les casiers sont un peu froids. Un cartable frotte le bois. Papa noue les lacets de Mila. Les lacets font un bruit de tissu. Tu as ton goûter dans la poche. Les lacets sont bien faits ? Oui, papa. Un cube jaune attend sur le tapis. Puis un cube bleu. Le tapis sent un peu la laine. En ce moment, Mila pose les cubes. Le cube jaune est lisse. Je fais une maison. Pour la voiture verte. Une maison au bout du tapis ? Oui. Elle doit arriver. Aniss arrive. Aniss parle peu. Il regarde le tapis. Mila a envie de poser beaucoup de questions. Elle referme un peu la bouche. On peut attendre. Tu peux tendre un jouet. La voiture verte est dans sa main. Les roues sont lisses. Aniss ne dit rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La fermeture du manteau rouge accroche un casier. Elle tient, papa. Tu la tires, Mila ? Oui, il est froid. Papa libère la fermeture, d'un coup. Une goutte saute sur la vitre. Elle est ronde. Tu as vu la goutte, Mila ? Oui, maman. La vitre est embuée, un peu. Mila pose un doigt au milieu. Un petit rond s'ouvre, net. Au bord, un &lt;emphasis level="moderate"&gt;éclat de rond&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, ce petit point ? Oui, un petit point. Les casiers sentent le bois mouillé. Ça sent la pluie, maman. Le goûter est dans la poche ? Oui, maman. Le bois du casier est froid, sous la paume. Il pique un peu. Tes doigts sont froids, Mila ? Un peu, papa. Un cube jaune attend sur le tapis. Puis un cube bleu, plus loin. Ils sont lisses. Le tapis est prêt, Mila ? Oui, papa. En ce moment, Mila pose les cubes. Je veux jouer à la voiture, maintenant ! Pour la maison, au bout du tapis. Une maison au bout du tapis ? Oui. Elle doit arriver tout de suite. La voiture verte est dans sa main. Les roues sont lisses, un peu froides. Aniss arrive près du tapis. Il s'arrête, sans parler. Tu viens, Aniss ? On fait la maison ? Tu prends la voiture ? Les questions tombent trop vite. Prends-la ! Mila tend la voiture trop vite. Aniss recule d'un pas. Ses épaules se serrent. Il ne dit rien. Aniss ? Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Mila ? Oui, papa. Tes mains tiennent la voiture, Mila ? Un peu, maman. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le petit rond, un instant. L'éclat de rond tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur la vitre.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Valentine est à l'école. Nino arrive. Nino parle peu. Il regarde le tapis. Valentine veut poser beaucoup de questions. Maman est venue avec elle ce matin. Maman dit doucement : on peut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. On n'imite pas. On ne va pas forcer la parole. Valentine prend une voiture. Elle va tendre un jouet. Elle tend la voiture vers Nino. Nino regarde. Il ne dit rien. Valentine attend. Nino prend la voiture. Il la fait rouler. Plus tard, au parc, Nino parle encore peu. Valentine se souvient. Elle attend. Elle va tendre un seau. On peut attendre. On peut tendre un jouet. On ne va pas forcer la parole. Nino pousse le seau. Valentine sourit. Maman dit : c'est possible de jouer avec peu de mots. [pause]</t>
+          <t>La fermeture du manteau rouge accroche un casier. Elle tient, papa. Tu la tires, Mila ? Oui, il est froid. Papa libère la fermeture, d'un coup. Une goutte saute sur la vitre. Elle est ronde. Tu as vu la goutte, Mila ? Oui, maman. La vitre est embuée, un peu. Mila pose un doigt au milieu. Un petit rond s'ouvre, net. Au bord, un &lt;emphasis&gt;éclat de rond&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, ce petit point ? Oui, un petit point. Les casiers sentent le bois mouillé. Ça sent la pluie, maman. Le goûter est dans la poche ? Oui, maman. Le bois du casier est froid, sous la paume. Il pique un peu. Tes doigts sont froids, Mila ? Un peu, papa. Un cube jaune attend sur le tapis. Puis un cube bleu, plus loin. Ils sont lisses. Le tapis est prêt, Mila ? Oui, papa. En ce moment, Mila pose les cubes. Je veux jouer à la voiture, maintenant ! Pour la maison, au bout du tapis. Une maison au bout du tapis ? Oui. Elle doit arriver tout de suite. La voiture verte est dans sa main. Les roues sont lisses, un peu froides. Aniss arrive près du tapis. Il s'arrête, sans parler. Tu viens, Aniss ? On fait la maison ? Tu prends la voiture ? Les questions tombent trop vite. Prends-la ! Mila tend la voiture trop vite. Aniss recule d'un pas. Ses épaules se serrent. Il ne dit rien. Aniss ? Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Aniss, Mila ? Oui, papa. Tes mains tiennent la voiture, Mila ? Un peu, maman. Mila refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le petit rond, un instant. L'éclat de rond tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur la vitre. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de rond</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,44 +1326,83 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_voiture_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une goutte tombe du manteau rouge.
-narrateur|Elle fait un rond sombre sur le carrelage.
-narrateur|Le manteau sent encore la pluie.
-narrateur|Les casiers sont un peu froids.
-narrateur|Un cartable frotte le bois.
-narrateur|Papa noue les lacets de Mila.
-narrateur|Les lacets font un bruit de tissu.
-maman|Tu as ton goûter dans la poche.
-papa|Les lacets sont bien faits ?
+          <t>narrateur|La fermeture du manteau rouge accroche un casier.
+enfant-f|Elle tient, papa.
+papa|Tu la tires, Mila ?
+enfant-f|Oui, il est froid.
+narrateur|Papa libère la fermeture, d'un coup.
+narrateur|Une goutte saute sur la vitre.
+enfant-f|Elle est ronde.
+maman|Tu as vu la goutte, Mila ?
+enfant-f|Oui, maman.
+narrateur|La vitre est embuée, un peu.
+narrateur|Mila pose un doigt au milieu.
+narrateur|Un petit rond s'ouvre, net.
+narrateur|Au bord, un éclat de rond brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, ce petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Les casiers sentent le bois mouillé.
+enfant-f|Ça sent la pluie, maman.
+maman|Le goûter est dans la poche ?
+enfant-f|Oui, maman.
+narrateur|Le bois du casier est froid, sous la paume.
+enfant-f|Il pique un peu.
+papa|Tes doigts sont froids, Mila ?
+enfant-f|Un peu, papa.
+narrateur|Un cube jaune attend sur le tapis.
+narrateur|Puis un cube bleu, plus loin.
+enfant-f|Ils sont lisses.
+papa|Le tapis est prêt, Mila ?
 enfant-f|Oui, papa.
-narrateur|Un cube jaune attend sur le tapis.
-narrateur|Puis un cube bleu.
-narrateur|Le tapis sent un peu la laine.
 narrateur|En ce moment, Mila pose les cubes.
-narrateur|Le cube jaune est lisse.
-enfant-f|Je fais une maison.
-enfant-f|Pour la voiture verte.
+enfant-f|Je veux jouer à la voiture, maintenant !
+enfant-f|Pour la maison, au bout du tapis.
 maman|Une maison au bout du tapis ?
 enfant-f|Oui.
-enfant-f|Elle doit arriver.
-narrateur|Aniss arrive.
-narrateur|Aniss parle peu.
-narrateur|Il regarde le tapis.
-narrateur|Mila a envie de poser beaucoup de questions.
-narrateur|Elle referme un peu la bouche.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
+enfant-f|Elle doit arriver tout de suite.
 narrateur|La voiture verte est dans sa main.
-narrateur|Les roues sont lisses.
-narrateur|Aniss ne dit rien.</t>
+narrateur|Les roues sont lisses, un peu froides.
+narrateur|Aniss arrive près du tapis.
+narrateur|Il s'arrête, sans parler.
+enfant-f|Tu viens, Aniss ?
+enfant-f|On fait la maison ?
+enfant-f|Tu prends la voiture ?
+narrateur|Les questions tombent trop vite.
+enfant-f|Prends-la !
+narrateur|Mila tend la voiture trop vite.
+narrateur|Aniss recule d'un pas.
+narrateur|Ses épaules se serrent.
+narrateur|Il ne dit rien.
+enfant-f|Aniss ?
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Aniss, Mila ?
+enfant-f|Oui, papa.
+maman|Tes mains tiennent la voiture, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le petit rond, un instant.
+narrateur|L'éclat de rond tremble, puis tient.
+enfant-f|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur la vitre.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>casiers,manteau</t>
         </is>
       </c>
     </row>
@@ -1395,12 +1434,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss parle peu. Que fait Mila ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss parle &lt;emphasis level="moderate"&gt;peu&lt;/emphasis&gt;. Que fait Mila ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Nino parle peu. Que fait Valentine ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss parle &lt;emphasis&gt;peu&lt;/emphasis&gt;. Que fait Mila ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1410,7 +1449,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>attendre | tendre un jouet | un jouet | la voiture | elle attend</t>
+          <t>attendre | tendre un jouet | un jouet | elle attend</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1463,7 +1502,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1471,10 +1510,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1489,34 +1528,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>peu</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1525,23 +1568,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=aniss_parle_peu_que_fait_mila; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1574,17 +1617,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila tend la voiture. Pour la maison. Elle attend. Un oiseau chante derrière la vitre. Aniss prend la voiture. Il la fait rouler. Les roues font un petit rrr. On ne force pas la parole. La voiture peut parler pour vous. Ils posent encore des cubes. Un toit. Un mur. Une porte. La maison a une porte. La voiture entre. Les roues s'arrêtent. Elle est arrivée. Aniss dit tout bas. Maison. Maison. Tu as su attendre. Bravo, Mila. Plus tard, au parc, le sable est frais. Papa s'assoit sur le banc. Le bois du banc est un peu froid. Aniss est là aussi. Il parle encore peu. Mila se souvient. Elle tend le seau bleu. Le seau est un peu rêche. Aniss le pousse. Un chemin de sable s'allonge. Il va jusqu'au bac. Chemin. Chemin.</t>
+          <t>Mila tend la voiture, sans se presser. Pour la maison. Elle attend, les mains ouvertes. Aniss ne dit rien. Il regarde les roues. Puis il avance un doigt. Il prend la voiture. Il la fait rouler, lentement. Les roues font un petit rrr. Elle roule. Tu entends les roues, Mila ? Oui, papa. La maison a un toit ? On pose un cube. Mila pose le jaune, sans se presser. Aniss pose le bleu, plus tard. Maison. Maison. La voiture entre sous le toit. Elle est arrivée. Elle est arrivée, Mila ? Oui, papa. Le ventre de Mila se desserre. Merci, Mila. Maman a vu les mains ouvertes. Le petit rond est sur la vitre ? Oui, papa. Un éclat de rond luit au bord. Il est là. Plus tard, ils vont au parc. Le sable, maman ? Le seau est dans le sac. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila tend la voiture. Pour la maison. Elle attend. Un oiseau chante derrière la vitre. Aniss prend la voiture. Il la fait rouler. Les roues font un petit rrr. On ne force pas la parole. La voiture peut parler pour vous. Ils posent encore des cubes. Un toit. Un mur. Une porte. La maison a une porte. La voiture entre. Les roues s'arrêtent. Elle est arrivée. Aniss dit tout bas. Maison. Maison. Tu as su attendre. Bravo, Mila. Plus tard, au parc, le sable est frais. Papa s'assoit sur le banc. Le bois du banc est un peu froid. Aniss est là aussi. Il parle encore peu. Mila se souvient. Elle tend le seau bleu. Le seau est un peu rêche. Aniss le pousse. Un chemin de sable s'allonge. Il va jusqu'au bac. Chemin. Chemin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila tend la voiture, sans se presser. Pour la maison. Elle &lt;emphasis level="moderate"&gt;attend&lt;/emphasis&gt;, les mains ouvertes. Aniss ne dit rien. Il regarde les roues. Puis il avance un doigt. Il prend la voiture. Il la fait rouler, lentement. Les roues font un petit rrr. Elle roule. Tu entends les roues, Mila ? Oui, papa. La maison a un toit ? On pose un cube. Mila pose le jaune, sans se presser. Aniss pose le bleu, plus tard. Maison. Maison. La voiture entre sous le toit. Elle est arrivée. Elle est arrivée, Mila ? Oui, papa. Le ventre de Mila se desserre. Merci, Mila. Maman a vu les mains ouvertes. Le petit rond est sur la vitre ? Oui, papa. Un éclat de rond luit au bord. Il est là. Plus tard, ils vont au parc. Le sable, maman ? Le seau est dans le sac. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Valentine a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Elle a tendu un jouet. Nino a pris la voiture. On n'a pas forcé la parole. [pause]</t>
+          <t>Mila tend la voiture, sans se presser. Pour la maison. Elle &lt;emphasis&gt;attend&lt;/emphasis&gt;, les mains ouvertes. Aniss ne dit rien. Il regarde les roues. Puis il avance un doigt. Il prend la voiture. Il la fait rouler, lentement. Les roues font un petit rrr. Elle roule. Tu entends les roues, Mila ? Oui, papa. La maison a un toit ? On pose un cube. Mila pose le jaune, sans se presser. Aniss pose le bleu, plus tard. Maison. Maison. La voiture entre sous le toit. Elle est arrivée. Elle est arrivée, Mila ? Oui, papa. Le ventre de Mila se desserre. Merci, Mila. Maman a vu les mains ouvertes. Le petit rond est sur la vitre ? Oui, papa. Un éclat de rond luit au bord. Il est là. Plus tard, ils vont au parc. Le sable, maman ? Le seau est dans le sac. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1631,7 +1674,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1639,10 +1682,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1665,30 +1708,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>attend</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1697,10 +1740,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1713,51 +1756,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_referme_la_bouche_tend_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila tend la voiture.
+          <t>narrateur|Mila tend la voiture, sans se presser.
 enfant-f|Pour la maison.
-narrateur|Elle attend.
-narrateur|Un oiseau chante derrière la vitre.
-narrateur|Aniss prend la voiture.
-narrateur|Il la fait rouler.
+narrateur|Elle attend, les mains ouvertes.
+narrateur|Aniss ne dit rien.
+narrateur|Il regarde les roues.
+narrateur|Puis il avance un doigt.
+narrateur|Il prend la voiture.
+narrateur|Il la fait rouler, lentement.
 narrateur|Les roues font un petit rrr.
-maman|On ne force pas la parole.
-papa|La voiture peut parler pour vous.
-narrateur|Ils posent encore des cubes.
-narrateur|Un toit.
-narrateur|Un mur.
-narrateur|Une porte.
-narrateur|La maison a une porte.
-narrateur|La voiture entre.
-narrateur|Les roues s'arrêtent.
+enfant-f|Elle roule.
+papa|Tu entends les roues, Mila ?
+enfant-f|Oui, papa.
+maman|La maison a un toit ?
+enfant-f|On pose un cube.
+narrateur|Mila pose le jaune, sans se presser.
+narrateur|Aniss pose le bleu, plus tard.
+copain|Maison.
+enfant-f|Maison.
+narrateur|La voiture entre sous le toit.
 enfant-f|Elle est arrivée.
-narrateur|Aniss dit tout bas.
-enfant-m|Maison.
-enfant-f|Maison.
-papa|Tu as su attendre.
-papa|Bravo, Mila.
-narrateur|Plus tard, au parc, le sable est frais.
-narrateur|Papa s'assoit sur le banc.
-narrateur|Le bois du banc est un peu froid.
-narrateur|Aniss est là aussi.
-narrateur|Il parle encore peu.
-narrateur|Mila se souvient.
-narrateur|Elle tend le seau bleu.
-narrateur|Le seau est un peu rêche.
-narrateur|Aniss le pousse.
-narrateur|Un chemin de sable s'allonge.
-narrateur|Il va jusqu'au bac.
-enfant-m|Chemin.
-enfant-f|Chemin.</t>
+papa|Elle est arrivée, Mila ?
+enfant-f|Oui, papa.
+narrateur|Le ventre de Mila se desserre.
+maman|Merci, Mila.
+narrateur|Maman a vu les mains ouvertes.
+papa|Le petit rond est sur la vitre ?
+enfant-f|Oui, papa.
+narrateur|Un éclat de rond luit au bord.
+enfant-f|Il est là.
+narrateur|Plus tard, ils vont au parc.
+enfant-f|Le sable, maman ?
+maman|Le seau est dans le sac.
+enfant-f|Oui, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>voiture,cubes</t>
         </is>
       </c>
     </row>
@@ -1784,17 +1825,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Aniss à mettre son manteau. Le manteau sent encore la pluie. Aniss fait un petit signe. À demain ? À demain. Le chemin reste dans le bac. Et la maison, à l'école. Deux arrivées, aujourd'hui. Le banc du parc reste vide. Une goutte sèche sur le carrelage, plus tard. Le manteau rouge ne goutte plus.</t>
+          <t>Le sable du parc est frais, sous les doigts. Il est froid, papa. Tu le sens, le sable ? Oui, papa. Mila tient le seau, trop près d'Aniss. On fait un chemin, maintenant ! Elle pousse le seau trop vite. Le sable s'envole un peu. Aniss recule, les épaules hautes. Oh. Mila refuse de foncer, cette fois. Elle referme la bouche. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le sable qui tombe. Elle revoit l'éclat de rond. Le seau, Aniss ? Aniss ne dit rien. Mila tend le seau, sans se presser. Elle attend. Aniss pousse le seau, tout seul. Un chemin de sable s'allonge. Chemin. Chemin. Le chemin va jusqu'au bac, Mila ? Oui, papa. Tes mains sont sablées, Mila ? Un peu, maman. Aniss souffle, longuement. Il a poussé, papa. Tu l'as vu, toi ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Aniss à mettre son manteau. Le manteau sent encore la pluie. Aniss fait un petit signe. À demain ? À demain. Le chemin reste dans le bac. Et la maison, à l'école. Deux arrivées, aujourd'hui. Le banc du parc reste vide. Une goutte sèche sur le carrelage, plus tard. Le manteau rouge ne goutte plus.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le sable du parc est frais, sous les doigts. Il est froid, papa. Tu le sens, le sable ? Oui, papa. Mila tient le seau, trop près d'Aniss. On fait un chemin, maintenant ! Elle pousse le seau trop vite. Le sable s'envole un peu. Aniss recule, les épaules hautes. Oh. Mila refuse de foncer, cette fois. Elle referme la bouche. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le sable qui tombe. Elle revoit l'&lt;emphasis level="moderate"&gt;éclat de rond&lt;/emphasis&gt;. Le seau, Aniss ? Aniss ne dit rien. Mila tend le seau, sans se presser. Elle attend. Aniss pousse le seau, tout seul. Un chemin de sable s'allonge. Chemin. Chemin. Le chemin va jusqu'au bac, Mila ? Oui, papa. Tes mains sont sablées, Mila ? Un peu, maman. Aniss souffle, longuement. Il a poussé, papa. Tu l'as vu, toi ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Nino à mettre son manteau. Nino fait un petit signe. Valentine dit : à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Le sable du parc est frais, sous les doigts. Il est froid, papa. Tu le sens, le sable ? Oui, papa. Mila tient le seau, trop près d'Aniss. On fait un chemin, maintenant ! Elle pousse le seau trop vite. Le sable s'envole un peu. Aniss recule, les épaules hautes. Oh. Mila refuse de foncer, cette fois. Elle referme la bouche. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le sable qui tombe. Elle revoit l'&lt;emphasis&gt;éclat de rond&lt;/emphasis&gt;. Le seau, Aniss ? Aniss ne dit rien. Mila tend le seau, sans se presser. Elle attend. Aniss pousse le seau, tout seul. Un chemin de sable s'allonge. Chemin. Chemin. Le chemin va jusqu'au bac, Mila ? Oui, papa. Tes mains sont sablées, Mila ? Un peu, maman. Aniss souffle, longuement. Il a poussé, papa. Tu l'as vu, toi ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1841,7 +1882,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1849,10 +1890,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1875,30 +1916,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de rond</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1907,10 +1948,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1921,20 +1962,51 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=seau_trop_vite_elle_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman aide Aniss à mettre son manteau.
-narrateur|Le manteau sent encore la pluie.
-narrateur|Aniss fait un petit signe.
-papa|À demain ?
-enfant-f|À demain.
-maman|Le chemin reste dans le bac.
-enfant-f|Et la maison, à l'école.
-papa|Deux arrivées, aujourd'hui.
-narrateur|Le banc du parc reste vide.
-narrateur|Une goutte sèche sur le carrelage, plus tard.
-narrateur|Le manteau rouge ne goutte plus.</t>
+          <t>narrateur|Le sable du parc est frais, sous les doigts.
+enfant-f|Il est froid, papa.
+papa|Tu le sens, le sable ?
+enfant-f|Oui, papa.
+narrateur|Mila tient le seau, trop près d'Aniss.
+enfant-f|On fait un chemin, maintenant !
+narrateur|Elle pousse le seau trop vite.
+narrateur|Le sable s'envole un peu.
+narrateur|Aniss recule, les épaules hautes.
+enfant-f|Oh.
+narrateur|Mila refuse de foncer, cette fois.
+narrateur|Elle referme la bouche.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le seau, un instant.
+narrateur|Elle écoute le sable qui tombe.
+narrateur|Elle revoit l'éclat de rond.
+enfant-f|Le seau, Aniss ?
+narrateur|Aniss ne dit rien.
+narrateur|Mila tend le seau, sans se presser.
+narrateur|Elle attend.
+narrateur|Aniss pousse le seau, tout seul.
+narrateur|Un chemin de sable s'allonge.
+copain|Chemin.
+enfant-f|Chemin.
+papa|Le chemin va jusqu'au bac, Mila ?
+enfant-f|Oui, papa.
+maman|Tes mains sont sablées, Mila ?
+enfant-f|Un peu, maman.
+narrateur|Aniss souffle, longuement.
+enfant-f|Il a poussé, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>sable,seau</t>
         </is>
       </c>
     </row>
@@ -1961,17 +2033,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La voiture est à la maison. Le seau a fait un chemin. Deux jeux, peu de mots.</t>
+          <t>Ils reviennent près des casiers. Le manteau est un peu sec, Mila ? Oui, maman. La maison reste au bout du tapis ? Oui, papa. La voiture verte dort sous le toit. Elle est arrivée. Maison. Le seau a fait un chemin. Deux jeux, Mila ? Oui, papa. Mila pose un doigt sur la vitre. Le petit rond est toujours là. Un éclat de rond tient au bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La voiture est à la maison. Le seau a fait un chemin. Deux jeux, peu de mots.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils reviennent près des casiers. Le manteau est un peu sec, Mila ? Oui, maman. La maison reste au bout du tapis ? Oui, papa. La voiture verte dort sous le toit. Elle est arrivée. Maison. Le seau a fait un chemin. Deux jeux, Mila ? Oui, papa. Mila pose un doigt sur la vitre. Le petit rond est toujours là. Un &lt;emphasis level="moderate"&gt;éclat de rond&lt;/emphasis&gt; tient au bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils reviennent près des casiers. Le manteau est un peu sec, Mila ? Oui, maman. La maison reste au bout du tapis ? Oui, papa. La voiture verte dort sous le toit. Elle est arrivée. Maison. Le seau a fait un chemin. Deux jeux, Mila ? Oui, papa. Mila pose un doigt sur la vitre. Le petit rond est toujours là. Un &lt;emphasis&gt;éclat de rond&lt;/emphasis&gt; tient au bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2018,15 +2090,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2038,12 +2110,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2052,17 +2124,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rond</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2071,11 +2147,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2084,26 +2160,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_au_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|La voiture est à la maison.
-maman|Le seau a fait un chemin.
-papa|Deux jeux, peu de mots.</t>
+          <t>narrateur|Ils reviennent près des casiers.
+maman|Le manteau est un peu sec, Mila ?
+enfant-f|Oui, maman.
+papa|La maison reste au bout du tapis ?
+enfant-f|Oui, papa.
+narrateur|La voiture verte dort sous le toit.
+enfant-f|Elle est arrivée.
+copain|Maison.
+enfant-f|Le seau a fait un chemin.
+papa|Deux jeux, Mila ?
+enfant-f|Oui, papa.
+narrateur|Mila pose un doigt sur la vitre.
+narrateur|Le petit rond est toujours là.
+narrateur|Un éclat de rond tient au bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>manteau,vitre</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2181,6 +2277,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>